<commit_message>
Deployed 3d65827 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/case_studies/outputs_cs1_r/results/CaseStudy_1_results.xlsx
+++ b/case_studies/outputs_cs1_r/results/CaseStudy_1_results.xlsx
@@ -32,10 +32,10 @@
     <t xml:space="preserve">age</t>
   </si>
   <si>
-    <t xml:space="preserve">65.38 ± 8.27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[45.00, 86.00]</t>
+    <t xml:space="preserve">65.30 ± 6.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[49.00, 82.00]</t>
   </si>
   <si>
     <t xml:space="preserve">sex</t>
@@ -50,37 +50,37 @@
     <t xml:space="preserve">criq</t>
   </si>
   <si>
-    <t xml:space="preserve">96.02 ± 11.34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[73.50, 120.10]</t>
+    <t xml:space="preserve">96.10 ± 11.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[74.00, 119.00]</t>
   </si>
   <si>
     <t xml:space="preserve">apacs</t>
   </si>
   <si>
-    <t xml:space="preserve">0.75 ± 0.07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[0.57, 0.88]</t>
+    <t xml:space="preserve">0.70 ± 0.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[0.39, 0.93]</t>
   </si>
   <si>
     <t xml:space="preserve">att_matr</t>
   </si>
   <si>
-    <t xml:space="preserve">36.88 ± 11.44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[5.00, 61.00]</t>
+    <t xml:space="preserve">31.95 ± 9.30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3.00, 48.00]</t>
   </si>
   <si>
     <t xml:space="preserve">moca</t>
   </si>
   <si>
-    <t xml:space="preserve">21.63 ± 6.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[8.17, 30.00]</t>
+    <t xml:space="preserve">21.73 ± 6.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[8.00, 30.00]</t>
   </si>
   <si>
     <t xml:space="preserve">n400_amp</t>
@@ -95,10 +95,10 @@
     <t xml:space="preserve">n400_lat</t>
   </si>
   <si>
-    <t xml:space="preserve">426.01 ± 14.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[402.10, 453.20]</t>
+    <t xml:space="preserve">426.25 ± 19.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[397.00, 460.10]</t>
   </si>
   <si>
     <t xml:space="preserve">p300_amp</t>
@@ -113,10 +113,10 @@
     <t xml:space="preserve">p300_lat</t>
   </si>
   <si>
-    <t xml:space="preserve">350.27 ± 18.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[313.60, 398.10]</t>
+    <t xml:space="preserve">400.63 ± 57.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[292.90, 553.70]</t>
   </si>
   <si>
     <t xml:space="preserve">Variable 1</t>
@@ -683,10 +683,10 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.327698627221405</v>
+        <v>-0.320769606504891</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0389976150383263</v>
+        <v>0.0435837846016806</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -700,10 +700,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.188309018221705</v>
+        <v>0.0287158250175099</v>
       </c>
       <c r="D3" t="n">
-        <v>0.244565274730857</v>
+        <v>0.860378822964118</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -717,10 +717,10 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.710048272978924</v>
+        <v>-0.442257377987873</v>
       </c>
       <c r="D4" t="n">
-        <v>0.000000287827957222292</v>
+        <v>0.00427181761439013</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -734,13 +734,13 @@
         <v>16</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.505856959409307</v>
+        <v>-0.206338803097071</v>
       </c>
       <c r="D5" t="n">
-        <v>0.000868683119733659</v>
+        <v>0.201454654612057</v>
       </c>
       <c r="E5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -751,10 +751,10 @@
         <v>19</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.283491592903718</v>
+        <v>-0.232971947710133</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0762831796642278</v>
+        <v>0.147977000388951</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -768,10 +768,10 @@
         <v>22</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.110962650001924</v>
+        <v>-0.105029229018177</v>
       </c>
       <c r="D7" t="n">
-        <v>0.495463228032329</v>
+        <v>0.518935561169763</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -785,10 +785,10 @@
         <v>25</v>
       </c>
       <c r="C8" t="n">
-        <v>0.180593965873249</v>
+        <v>0.0775624370636242</v>
       </c>
       <c r="D8" t="n">
-        <v>0.264782854938057</v>
+        <v>0.634280712550793</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -802,10 +802,10 @@
         <v>28</v>
       </c>
       <c r="C9" t="n">
-        <v>0.151630607886565</v>
+        <v>0.157183743081252</v>
       </c>
       <c r="D9" t="n">
-        <v>0.350302679495509</v>
+        <v>0.332728491688458</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -819,10 +819,10 @@
         <v>31</v>
       </c>
       <c r="C10" t="n">
-        <v>0.502322204253447</v>
+        <v>0.426480273108518</v>
       </c>
       <c r="D10" t="n">
-        <v>0.000956916848281542</v>
+        <v>0.00606603871637525</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -836,13 +836,13 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.317113758018998</v>
+        <v>0.249752434334393</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0461741969850418</v>
+        <v>0.120129373526373</v>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -853,10 +853,10 @@
         <v>13</v>
       </c>
       <c r="C12" t="n">
-        <v>0.211748718386119</v>
+        <v>0.103537942979161</v>
       </c>
       <c r="D12" t="n">
-        <v>0.189627587343053</v>
+        <v>0.524920444889512</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -870,10 +870,10 @@
         <v>16</v>
       </c>
       <c r="C13" t="n">
-        <v>0.241321184370394</v>
+        <v>0.174162717116873</v>
       </c>
       <c r="D13" t="n">
-        <v>0.133582659195186</v>
+        <v>0.282458060849275</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -887,10 +887,10 @@
         <v>19</v>
       </c>
       <c r="C14" t="n">
-        <v>0.235535514436143</v>
+        <v>0.223489474691197</v>
       </c>
       <c r="D14" t="n">
-        <v>0.143441427888717</v>
+        <v>0.165668484242298</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -921,10 +921,10 @@
         <v>25</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.0463724570110574</v>
+        <v>-0.00844938876332995</v>
       </c>
       <c r="D16" t="n">
-        <v>0.776304666229273</v>
+        <v>0.958731918637052</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -955,10 +955,10 @@
         <v>31</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.371295914920262</v>
+        <v>-0.354588210575591</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0183324388039996</v>
+        <v>0.024767838506102</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -972,13 +972,13 @@
         <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>0.35673609029997</v>
+        <v>0.222004687070825</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0238478752059597</v>
+        <v>0.168571319800999</v>
       </c>
       <c r="E19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -989,10 +989,10 @@
         <v>16</v>
       </c>
       <c r="C20" t="n">
-        <v>0.503610873376333</v>
+        <v>0.55884482093072</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0009238676796106</v>
+        <v>0.000178242644795936</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -1006,10 +1006,10 @@
         <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>0.218572076981164</v>
+        <v>0.162032176830416</v>
       </c>
       <c r="D21" t="n">
-        <v>0.175422131958076</v>
+        <v>0.317839995573332</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -1023,10 +1023,10 @@
         <v>22</v>
       </c>
       <c r="C22" t="n">
-        <v>0.0354430134475999</v>
+        <v>0.00332743172689629</v>
       </c>
       <c r="D22" t="n">
-        <v>0.828113853176359</v>
+        <v>0.983742442744649</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -1040,10 +1040,10 @@
         <v>25</v>
       </c>
       <c r="C23" t="n">
-        <v>-0.270666299275654</v>
+        <v>-0.242403711075757</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0911702560382486</v>
+        <v>0.131795342246067</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -1057,13 +1057,13 @@
         <v>28</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.313757021739211</v>
+        <v>-0.285460033134095</v>
       </c>
       <c r="D24" t="n">
-        <v>0.048660912245745</v>
+        <v>0.0741774278127727</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1074,10 +1074,10 @@
         <v>31</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.303315968550147</v>
+        <v>-0.209461070728193</v>
       </c>
       <c r="D25" t="n">
-        <v>0.057092577416315</v>
+        <v>0.194567389683841</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -1091,13 +1091,13 @@
         <v>16</v>
       </c>
       <c r="C26" t="n">
-        <v>0.446456418227507</v>
+        <v>0.225905338427392</v>
       </c>
       <c r="D26" t="n">
-        <v>0.00388034762724634</v>
+        <v>0.161022782903692</v>
       </c>
       <c r="E26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1108,10 +1108,10 @@
         <v>19</v>
       </c>
       <c r="C27" t="n">
-        <v>0.193628521063276</v>
+        <v>0.0795512667081346</v>
       </c>
       <c r="D27" t="n">
-        <v>0.231247446771512</v>
+        <v>0.625587524059061</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1125,10 +1125,10 @@
         <v>22</v>
       </c>
       <c r="C28" t="n">
-        <v>0.345011180780759</v>
+        <v>0.40310559697844</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0292362923048999</v>
+        <v>0.00990633583670473</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -1142,10 +1142,10 @@
         <v>25</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.459624693214568</v>
+        <v>-0.651391520347971</v>
       </c>
       <c r="D29" t="n">
-        <v>0.00284806149662708</v>
+        <v>0.00000531154035994955</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -1159,10 +1159,10 @@
         <v>28</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.141595274016141</v>
+        <v>-0.0488045674558732</v>
       </c>
       <c r="D30" t="n">
-        <v>0.383463242520514</v>
+        <v>0.764896100157228</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1176,10 +1176,10 @@
         <v>31</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.468611764659109</v>
+        <v>-0.343487027264936</v>
       </c>
       <c r="D31" t="n">
-        <v>0.00228989446758346</v>
+        <v>0.0300053262350475</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -1193,10 +1193,10 @@
         <v>19</v>
       </c>
       <c r="C32" t="n">
-        <v>0.278468492621404</v>
+        <v>0.204463305321157</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0818689175462257</v>
+        <v>0.205672830253927</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1210,10 +1210,10 @@
         <v>22</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.0361345223533805</v>
+        <v>-0.0894587013783039</v>
       </c>
       <c r="D33" t="n">
-        <v>0.82481203335059</v>
+        <v>0.583041085601619</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1227,10 +1227,10 @@
         <v>25</v>
       </c>
       <c r="C34" t="n">
-        <v>-0.24457185102238</v>
+        <v>-0.224429054194273</v>
       </c>
       <c r="D34" t="n">
-        <v>0.128269194837893</v>
+        <v>0.163850309204321</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1244,10 +1244,10 @@
         <v>28</v>
       </c>
       <c r="C35" t="n">
-        <v>0.330176679631824</v>
+        <v>0.376248620286081</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0374562195083798</v>
+        <v>0.0167197588081529</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -1261,10 +1261,10 @@
         <v>31</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.462716275600186</v>
+        <v>-0.34354988008823</v>
       </c>
       <c r="D36" t="n">
-        <v>0.00264390586769209</v>
+        <v>0.0299732863725055</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -1278,10 +1278,10 @@
         <v>22</v>
       </c>
       <c r="C37" t="n">
-        <v>0.122715019978909</v>
+        <v>0.115715691190831</v>
       </c>
       <c r="D37" t="n">
-        <v>0.450629936986069</v>
+        <v>0.47706108219202</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1295,10 +1295,10 @@
         <v>25</v>
       </c>
       <c r="C38" t="n">
-        <v>-0.0104890295424188</v>
+        <v>0.0266884895999619</v>
       </c>
       <c r="D38" t="n">
-        <v>0.948781874753659</v>
+        <v>0.870148869059894</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1312,10 +1312,10 @@
         <v>28</v>
       </c>
       <c r="C39" t="n">
-        <v>-0.173742710318284</v>
+        <v>-0.173035316464961</v>
       </c>
       <c r="D39" t="n">
-        <v>0.283638464511282</v>
+        <v>0.285633789874221</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1329,10 +1329,10 @@
         <v>31</v>
       </c>
       <c r="C40" t="n">
-        <v>-0.177798717194351</v>
+        <v>-0.125673792959967</v>
       </c>
       <c r="D40" t="n">
-        <v>0.272373058647029</v>
+        <v>0.439701240872935</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1346,10 +1346,10 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>-0.00600992842132089</v>
+        <v>0.00685515170120411</v>
       </c>
       <c r="D41" t="n">
-        <v>0.970640397110013</v>
+        <v>0.966513510782646</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1380,10 +1380,10 @@
         <v>31</v>
       </c>
       <c r="C43" t="n">
-        <v>-0.283234380296387</v>
+        <v>-0.284521046729093</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0765617563325248</v>
+        <v>0.0751761540880915</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1397,10 +1397,10 @@
         <v>28</v>
       </c>
       <c r="C44" t="n">
-        <v>-0.121129158741956</v>
+        <v>-0.138175260589881</v>
       </c>
       <c r="D44" t="n">
-        <v>0.456547772335329</v>
+        <v>0.395172134291675</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1414,10 +1414,10 @@
         <v>31</v>
       </c>
       <c r="C45" t="n">
-        <v>0.185185896980399</v>
+        <v>0.131439968951615</v>
       </c>
       <c r="D45" t="n">
-        <v>0.252620406539266</v>
+        <v>0.41882855161098</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1431,10 +1431,10 @@
         <v>31</v>
       </c>
       <c r="C46" t="n">
-        <v>-0.012792214140414</v>
+        <v>-0.0279148869828427</v>
       </c>
       <c r="D46" t="n">
-        <v>0.937555463480605</v>
+        <v>0.864236300375781</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1485,19 +1485,19 @@
         <v>46</v>
       </c>
       <c r="C2" t="n">
-        <v>1.7627319133453</v>
+        <v>2.73381068650082</v>
       </c>
       <c r="D2" t="n">
-        <v>0.200112869875774</v>
+        <v>0.275566133710444</v>
       </c>
       <c r="E2" t="n">
-        <v>0.000000000164246891895972</v>
+        <v>0.00000000000768147362157142</v>
       </c>
       <c r="F2" t="n">
-        <v>1.37051789554583</v>
+        <v>2.1937109890694</v>
       </c>
       <c r="G2" t="n">
-        <v>2.15494593114476</v>
+        <v>3.27391038393224</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -1511,19 +1511,19 @@
         <v>25</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.0017301359723672</v>
+        <v>-0.0041681845826491</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000469494035794115</v>
+        <v>0.000594789975551529</v>
       </c>
       <c r="E3" t="n">
-        <v>0.000747269424157931</v>
+        <v>0.0000000320612999898688</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.00265032737348002</v>
+        <v>-0.00533395151309556</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.000809944571254373</v>
+        <v>-0.00300241765220265</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1537,19 +1537,19 @@
         <v>22</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0231799821449598</v>
+        <v>0.0548452087434151</v>
       </c>
       <c r="D4" t="n">
-        <v>0.00786014804587281</v>
+        <v>0.0132785741862392</v>
       </c>
       <c r="E4" t="n">
-        <v>0.00557005176614627</v>
+        <v>0.000205719480977326</v>
       </c>
       <c r="F4" t="n">
-        <v>0.00777437506189619</v>
+        <v>0.0288196815723431</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0385855892280234</v>
+        <v>0.0808707359144871</v>
       </c>
       <c r="H4" t="b">
         <v>1</v>
@@ -1563,19 +1563,19 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.00551327026002523</v>
+        <v>-0.00693536773944796</v>
       </c>
       <c r="D5" t="n">
-        <v>0.000845497896766319</v>
+        <v>0.00175696906993948</v>
       </c>
       <c r="E5" t="n">
-        <v>0.000000140783075270525</v>
+        <v>0.0003514613978269</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.00717041568669158</v>
+        <v>-0.0103789638384802</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.00385612483335888</v>
+        <v>-0.00349177164041574</v>
       </c>
       <c r="H5" t="b">
         <v>1</v>
@@ -1589,19 +1589,19 @@
         <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>-38.056536590148</v>
+        <v>-51.6522978349967</v>
       </c>
       <c r="D6" t="n">
-        <v>47.0289454331225</v>
+        <v>27.6238737520133</v>
       </c>
       <c r="E6" t="n">
-        <v>0.424367633140491</v>
+        <v>0.0706788082754439</v>
       </c>
       <c r="F6" t="n">
-        <v>-130.231575869968</v>
+        <v>-105.794095502424</v>
       </c>
       <c r="G6" t="n">
-        <v>54.1185026896717</v>
+        <v>2.48949983243076</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1615,19 +1615,19 @@
         <v>31</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.0459565793252</v>
+        <v>-0.0108225862020003</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0730069393664283</v>
+        <v>0.0182680449197135</v>
       </c>
       <c r="E7" t="n">
-        <v>0.533502140177102</v>
+        <v>0.557724346845375</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.189047551104899</v>
+        <v>-0.0466272963125986</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0971343924544989</v>
+        <v>0.0249821239085981</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -1641,19 +1641,19 @@
         <v>28</v>
       </c>
       <c r="C8" t="n">
-        <v>3.83371356654628</v>
+        <v>3.37629648016998</v>
       </c>
       <c r="D8" t="n">
-        <v>0.643971140278157</v>
+        <v>0.536885518630549</v>
       </c>
       <c r="E8" t="n">
-        <v>0.00000124280341749202</v>
+        <v>0.000000471841477305291</v>
       </c>
       <c r="F8" t="n">
-        <v>2.5715533245179</v>
+        <v>2.32402019983299</v>
       </c>
       <c r="G8" t="n">
-        <v>5.09587380857466</v>
+        <v>4.42857276050696</v>
       </c>
       <c r="H8" t="b">
         <v>1</v>
@@ -1667,19 +1667,19 @@
         <v>25</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0704651515681286</v>
+        <v>0.0402143605088182</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0738288268009405</v>
+        <v>0.0460402569889754</v>
       </c>
       <c r="E9" t="n">
-        <v>0.347016051496178</v>
+        <v>0.388919790581151</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0742366899825603</v>
+        <v>-0.0500228850285421</v>
       </c>
       <c r="G9" t="n">
-        <v>0.215166993118818</v>
+        <v>0.130451606046178</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -1693,19 +1693,19 @@
         <v>22</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.678295132068312</v>
+        <v>-0.641793314754469</v>
       </c>
       <c r="D10" t="n">
-        <v>1.22775756723874</v>
+        <v>1.02222642767812</v>
       </c>
       <c r="E10" t="n">
-        <v>0.584467322970707</v>
+        <v>0.534564802137903</v>
       </c>
       <c r="F10" t="n">
-        <v>-3.08465574560275</v>
+        <v>-2.64532029704862</v>
       </c>
       <c r="G10" t="n">
-        <v>1.72806548146612</v>
+        <v>1.36173366753968</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1719,19 +1719,19 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.658099876728523</v>
+        <v>-0.455266606089481</v>
       </c>
       <c r="D11" t="n">
-        <v>0.146921634608142</v>
+        <v>0.149828345679595</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0000896116989071058</v>
+        <v>0.00470614500869738</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.946060989110235</v>
+        <v>-0.748924767484705</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.370138764346812</v>
+        <v>-0.161608444694257</v>
       </c>
       <c r="H11" t="b">
         <v>1</v>
@@ -1745,19 +1745,19 @@
         <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.676134460180054</v>
+        <v>-0.618947605418479</v>
       </c>
       <c r="D12" t="n">
-        <v>2.26044859478304</v>
+        <v>1.87509034896077</v>
       </c>
       <c r="E12" t="n">
-        <v>0.766786248112779</v>
+        <v>0.74348366821566</v>
       </c>
       <c r="F12" t="n">
-        <v>-5.10653229485899</v>
+        <v>-4.29405715714023</v>
       </c>
       <c r="G12" t="n">
-        <v>3.75426337449888</v>
+        <v>3.05616194630327</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -1771,19 +1771,19 @@
         <v>10</v>
       </c>
       <c r="C13" t="n">
-        <v>0.619492104047858</v>
+        <v>0.639508701902286</v>
       </c>
       <c r="D13" t="n">
-        <v>0.106035271464649</v>
+        <v>0.0882179516300428</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00000171414988468569</v>
+        <v>0.0000000309232781279285</v>
       </c>
       <c r="F13" t="n">
-        <v>0.411666790886218</v>
+        <v>0.466604693917506</v>
       </c>
       <c r="G13" t="n">
-        <v>0.827317417209498</v>
+        <v>0.812412709887067</v>
       </c>
       <c r="H13" t="b">
         <v>1</v>
@@ -1797,22 +1797,22 @@
         <v>46</v>
       </c>
       <c r="C14" t="n">
-        <v>-24.4865176885144</v>
+        <v>-39.836264060861</v>
       </c>
       <c r="D14" t="n">
-        <v>15.389746129674</v>
+        <v>12.3967314751085</v>
       </c>
       <c r="E14" t="n">
-        <v>0.120333002185403</v>
+        <v>0.00276517985106481</v>
       </c>
       <c r="F14" t="n">
-        <v>-54.64986583389</v>
+        <v>-64.1334112780877</v>
       </c>
       <c r="G14" t="n">
-        <v>5.67683045686125</v>
+        <v>-15.5391168436343</v>
       </c>
       <c r="H14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1823,19 +1823,19 @@
         <v>28</v>
       </c>
       <c r="C15" t="n">
-        <v>3.81968429896233</v>
+        <v>3.37819090822344</v>
       </c>
       <c r="D15" t="n">
-        <v>0.580570494904684</v>
+        <v>0.482593783141242</v>
       </c>
       <c r="E15" t="n">
-        <v>0.000000117780154812583</v>
+        <v>0.0000000328209471888635</v>
       </c>
       <c r="F15" t="n">
-        <v>2.68178703846255</v>
+        <v>2.43232447410367</v>
       </c>
       <c r="G15" t="n">
-        <v>4.9575815594621</v>
+        <v>4.3240573423432</v>
       </c>
       <c r="H15" t="b">
         <v>1</v>
@@ -1849,19 +1849,19 @@
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.667928483901455</v>
+        <v>-0.461561249760049</v>
       </c>
       <c r="D16" t="n">
-        <v>0.120148270063826</v>
+        <v>0.123495924363125</v>
       </c>
       <c r="E16" t="n">
-        <v>0.00000269928079111594</v>
+        <v>0.000643673318690692</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.903414766031346</v>
+        <v>-0.703608813749258</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.432442201771564</v>
+        <v>-0.219513685770841</v>
       </c>
       <c r="H16" t="b">
         <v>1</v>
@@ -1875,19 +1875,19 @@
         <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>0.603333927445159</v>
+        <v>0.627177611815129</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0912023504198029</v>
+        <v>0.0756625208579822</v>
       </c>
       <c r="E17" t="n">
-        <v>0.00000010549016168614</v>
+        <v>0.0000000007246298232408</v>
       </c>
       <c r="F17" t="n">
-        <v>0.424580605316944</v>
+        <v>0.478881795953974</v>
       </c>
       <c r="G17" t="n">
-        <v>0.782087249573374</v>
+        <v>0.775473427676285</v>
       </c>
       <c r="H17" t="b">
         <v>1</v>
@@ -1917,7 +1917,7 @@
         <v>28</v>
       </c>
       <c r="B2" t="n">
-        <v>1.12022646945821</v>
+        <v>1.12215922462642</v>
       </c>
     </row>
     <row r="3">
@@ -1925,7 +1925,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>1.04707714548854</v>
+        <v>1.03156798230141</v>
       </c>
     </row>
     <row r="4">
@@ -1933,7 +1933,7 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>1.13470745145541</v>
+        <v>1.09533755448983</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed c44c7d6 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/case_studies/outputs_cs1_r/results/CaseStudy_1_results.xlsx
+++ b/case_studies/outputs_cs1_r/results/CaseStudy_1_results.xlsx
@@ -720,7 +720,7 @@
         <v>-0.442257377987873</v>
       </c>
       <c r="D4" t="n">
-        <v>0.00427181761439013</v>
+        <v>0.0042718176143901</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -822,7 +822,7 @@
         <v>0.426480273108518</v>
       </c>
       <c r="D10" t="n">
-        <v>0.00606603871637525</v>
+        <v>0.00606603871637527</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -958,7 +958,7 @@
         <v>-0.354588210575591</v>
       </c>
       <c r="D18" t="n">
-        <v>0.024767838506102</v>
+        <v>0.0247678385061021</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -1023,7 +1023,7 @@
         <v>22</v>
       </c>
       <c r="C22" t="n">
-        <v>0.00332743172689629</v>
+        <v>0.00332743172689628</v>
       </c>
       <c r="D22" t="n">
         <v>0.983742442744649</v>
@@ -1060,7 +1060,7 @@
         <v>-0.285460033134095</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0741774278127727</v>
+        <v>0.0741774278127728</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -1094,7 +1094,7 @@
         <v>0.225905338427392</v>
       </c>
       <c r="D26" t="n">
-        <v>0.161022782903692</v>
+        <v>0.161022782903693</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1159,7 +1159,7 @@
         <v>28</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.0488045674558732</v>
+        <v>-0.0488045674558731</v>
       </c>
       <c r="D30" t="n">
         <v>0.764896100157228</v>
@@ -1179,7 +1179,7 @@
         <v>-0.343487027264936</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0300053262350475</v>
+        <v>0.0300053262350476</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -1281,7 +1281,7 @@
         <v>0.115715691190831</v>
       </c>
       <c r="D37" t="n">
-        <v>0.47706108219202</v>
+        <v>0.477061082192021</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1298,7 +1298,7 @@
         <v>0.0266884895999619</v>
       </c>
       <c r="D38" t="n">
-        <v>0.870148869059894</v>
+        <v>0.870148869059895</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1315,7 +1315,7 @@
         <v>-0.173035316464961</v>
       </c>
       <c r="D39" t="n">
-        <v>0.285633789874221</v>
+        <v>0.285633789874222</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1346,7 +1346,7 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>0.00685515170120411</v>
+        <v>0.0068551517012041</v>
       </c>
       <c r="D41" t="n">
         <v>0.966513510782646</v>
@@ -1417,7 +1417,7 @@
         <v>0.131439968951615</v>
       </c>
       <c r="D45" t="n">
-        <v>0.41882855161098</v>
+        <v>0.418828551610981</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1491,13 +1491,13 @@
         <v>0.275566133710444</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00000000000768147362157142</v>
+        <v>0.00000000000768147362157145</v>
       </c>
       <c r="F2" t="n">
         <v>2.1937109890694</v>
       </c>
       <c r="G2" t="n">
-        <v>3.27391038393224</v>
+        <v>3.27391038393223</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -1514,16 +1514,16 @@
         <v>-0.0041681845826491</v>
       </c>
       <c r="D3" t="n">
-        <v>0.000594789975551529</v>
+        <v>0.000594789975551528</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0000000320612999898688</v>
+        <v>0.0000000320612999898691</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.00533395151309556</v>
+        <v>-0.00533395151309555</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.00300241765220265</v>
+        <v>-0.00300241765220264</v>
       </c>
       <c r="H3" t="b">
         <v>1</v>
@@ -1543,7 +1543,7 @@
         <v>0.0132785741862392</v>
       </c>
       <c r="E4" t="n">
-        <v>0.000205719480977326</v>
+        <v>0.000205719480977325</v>
       </c>
       <c r="F4" t="n">
         <v>0.0288196815723431</v>
@@ -1563,13 +1563,13 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.00693536773944796</v>
+        <v>-0.00693536773944795</v>
       </c>
       <c r="D5" t="n">
         <v>0.00175696906993948</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0003514613978269</v>
+        <v>0.000351461397826905</v>
       </c>
       <c r="F5" t="n">
         <v>-0.0103789638384802</v>
@@ -1595,13 +1595,13 @@
         <v>27.6238737520133</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0706788082754439</v>
+        <v>0.0706788082754436</v>
       </c>
       <c r="F6" t="n">
         <v>-105.794095502424</v>
       </c>
       <c r="G6" t="n">
-        <v>2.48949983243076</v>
+        <v>2.4894998324307</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1644,10 +1644,10 @@
         <v>3.37629648016998</v>
       </c>
       <c r="D8" t="n">
-        <v>0.536885518630549</v>
+        <v>0.536885518630548</v>
       </c>
       <c r="E8" t="n">
-        <v>0.000000471841477305291</v>
+        <v>0.000000471841477305286</v>
       </c>
       <c r="F8" t="n">
         <v>2.32402019983299</v>
@@ -1670,13 +1670,13 @@
         <v>0.0402143605088182</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0460402569889754</v>
+        <v>0.0460402569889753</v>
       </c>
       <c r="E9" t="n">
         <v>0.388919790581151</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.0500228850285421</v>
+        <v>-0.050022885028542</v>
       </c>
       <c r="G9" t="n">
         <v>0.130451606046178</v>
@@ -1693,7 +1693,7 @@
         <v>22</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.641793314754469</v>
+        <v>-0.641793314754468</v>
       </c>
       <c r="D10" t="n">
         <v>1.02222642767812</v>
@@ -1725,7 +1725,7 @@
         <v>0.149828345679595</v>
       </c>
       <c r="E11" t="n">
-        <v>0.00470614500869738</v>
+        <v>0.00470614500869739</v>
       </c>
       <c r="F11" t="n">
         <v>-0.748924767484705</v>
@@ -1745,13 +1745,13 @@
         <v>7</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.618947605418479</v>
+        <v>-0.618947605418482</v>
       </c>
       <c r="D12" t="n">
         <v>1.87509034896077</v>
       </c>
       <c r="E12" t="n">
-        <v>0.74348366821566</v>
+        <v>0.743483668215658</v>
       </c>
       <c r="F12" t="n">
         <v>-4.29405715714023</v>
@@ -1803,13 +1803,13 @@
         <v>12.3967314751085</v>
       </c>
       <c r="E14" t="n">
-        <v>0.00276517985106481</v>
+        <v>0.00276517985106484</v>
       </c>
       <c r="F14" t="n">
         <v>-64.1334112780877</v>
       </c>
       <c r="G14" t="n">
-        <v>-15.5391168436343</v>
+        <v>-15.5391168436342</v>
       </c>
       <c r="H14" t="b">
         <v>1</v>
@@ -1878,10 +1878,10 @@
         <v>0.627177611815129</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0756625208579822</v>
+        <v>0.0756625208579821</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0000000007246298232408</v>
+        <v>0.000000000724629823240795</v>
       </c>
       <c r="F17" t="n">
         <v>0.478881795953974</v>

</xml_diff>